<commit_message>
feat(access): adiciona seed inicial de usuários locais para operação do EVOLV
</commit_message>
<xml_diff>
--- a/Banco Piperun.xlsx
+++ b/Banco Piperun.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1d87dc2f7073ca7b/Área de Trabalho/PROJETOS DIGITAIS/Evolv/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{ADA6A1B4-7CCB-4E0B-B79A-4B0E775FE2B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{ADA6A1B4-7CCB-4E0B-B79A-4B0E775FE2B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6254C6AA-7019-4465-832B-045FF9E313FC}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -6791,11 +6791,31 @@
   <dimension ref="A1:Y764"/>
   <sheetFormatPr defaultColWidth="11.19921875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="36.69921875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="13.296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="36.09765625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="30.19921875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.09765625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="24.8984375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="28.59765625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.59765625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.19921875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.09765625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="73.59765625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.796875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.3984375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="7.296875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="8" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="13.09765625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="30.296875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="22.296875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="13.8984375" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="21.19921875" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="29.19921875" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="24.8984375" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="16.796875" bestFit="1" customWidth="1"/>
     <col min="24" max="24" width="41.5" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="38.69921875" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="38.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:25" x14ac:dyDescent="0.3">

</xml_diff>